<commit_message>
- Merge Option update
</commit_message>
<xml_diff>
--- a/rs/src/tests/TestFiles/merge.xlsx
+++ b/rs/src/tests/TestFiles/merge.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\draviavemal\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0D489C8-93DA-47DC-8A18-80BC47C3BD77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED79003D-52F5-4FAB-930A-0F2189C64611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2B274876-FCAD-4C87-B4D3-71831F56BCE5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{2B274876-FCAD-4C87-B4D3-71831F56BCE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="edit" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
   <si>
     <t>Merge 1</t>
   </si>
@@ -45,9 +46,6 @@
     <t>Merge 3</t>
   </si>
   <si>
-    <t>Merge 4 with rape the text content</t>
-  </si>
-  <si>
     <t>Merge Top Left</t>
   </si>
   <si>
@@ -61,6 +59,12 @@
   </si>
   <si>
     <t>Link</t>
+  </si>
+  <si>
+    <t>Merge 4 with wrap the text content</t>
+  </si>
+  <si>
+    <t>Merge 2 Delete this</t>
   </si>
 </sst>
 </file>
@@ -109,6 +113,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -116,9 +123,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -442,131 +446,131 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="J3" s="2" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="J3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="J7" s="3" t="s">
+      <c r="G7" s="3"/>
+      <c r="J7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+    </row>
+    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+    </row>
+    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+    </row>
+    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+    </row>
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="N12" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-    </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-    </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-    </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="N12" s="4" t="s">
+      <c r="O12" s="5"/>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+    </row>
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+    </row>
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+    </row>
+    <row r="20" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J20" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="O12" s="4"/>
-    </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
-    </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-    </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
-    </row>
-    <row r="20" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J20" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
     </row>
     <row r="21" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
     </row>
     <row r="22" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
     </row>
     <row r="23" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
     </row>
     <row r="24" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
     </row>
     <row r="25" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
     </row>
     <row r="34" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C34" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E38" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -584,4 +588,158 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEBFA7E2-E448-4110-995C-1DD3C1E05CDA}">
+  <dimension ref="B2:P38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="J3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+    </row>
+    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+    </row>
+    <row r="7" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="J7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+    </row>
+    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+    </row>
+    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+    </row>
+    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+    </row>
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="N12" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="O12" s="5"/>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+    </row>
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+    </row>
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+    </row>
+    <row r="20" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J20" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+    </row>
+    <row r="21" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+    </row>
+    <row r="22" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+    </row>
+    <row r="23" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+    </row>
+    <row r="24" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+    </row>
+    <row r="25" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
+    </row>
+    <row r="34" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C34" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E38" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B2:D4"/>
+    <mergeCell ref="J3:P3"/>
+    <mergeCell ref="F7:G14"/>
+    <mergeCell ref="J7:L9"/>
+    <mergeCell ref="N12:O15"/>
+    <mergeCell ref="J20:L25"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C34" r:id="rId1" xr:uid="{4D4BC2A7-F6C1-4FA6-95CA-BC7601928FCF}"/>
+    <hyperlink ref="E38:F38" r:id="rId2" display="multiple" xr:uid="{175BA9E8-0128-403F-9F6B-569187684E43}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>